<commit_message>
Przebuduj okładki według rodzaju opracowania
</commit_message>
<xml_diff>
--- a/KONSPEKT - ŚWIĄTECZNE.xlsx
+++ b/KONSPEKT - ŚWIĄTECZNE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DYSK GOOGLE\[PATRONITE] - MATERIAŁY WORD I PDF\HTML - UTWORY ŚWIĄTECZNE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6292CECF-A05D-4C38-93F0-CC9CFA48ABED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15C20B6-E5FD-4371-90C7-574B4E6638F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13305" yWindow="0" windowWidth="25200" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BAZA" sheetId="1" r:id="rId1"/>
@@ -25,15 +25,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="127">
   <si>
     <t>UTWÓR</t>
   </si>
   <si>
+    <t>POZIOM</t>
+  </si>
+  <si>
+    <t>RODZAJ OPRACOWANIA</t>
+  </si>
+  <si>
+    <t>YOUTUBE</t>
+  </si>
+  <si>
     <t>WYKONAWCA</t>
   </si>
   <si>
-    <t>POZIOM</t>
+    <t>KATEGORIE DODATKOWE</t>
+  </si>
+  <si>
+    <t>LINK DO DYSKU</t>
   </si>
   <si>
     <t>OPIS</t>
@@ -42,25 +54,13 @@
     <t>TAGI</t>
   </si>
   <si>
-    <t>RODZAJ OPRACOWANIA</t>
-  </si>
-  <si>
-    <t>KATEGORIE DODATKOWE</t>
-  </si>
-  <si>
-    <t>YOUTUBE</t>
-  </si>
-  <si>
-    <t>LINK DO DYSKU</t>
-  </si>
-  <si>
     <t>DATA</t>
   </si>
   <si>
     <t>Aniołek Maleńki</t>
   </si>
   <si>
-    <t>MELODIA / SOLO LINE</t>
+    <t>BANALNY</t>
   </si>
   <si>
     <t>ŚWIĄTECZNE</t>
@@ -72,6 +72,9 @@
     <t>Aniołek Maleńki D Dur</t>
   </si>
   <si>
+    <t>ŚREDNI</t>
+  </si>
+  <si>
     <t>AKORDY</t>
   </si>
   <si>
@@ -87,12 +90,12 @@
     <t>https://drive.google.com/drive/folders/1dzvyj3rM4bXOstn2XjcDJUCTCqxHJfma</t>
   </si>
   <si>
-    <t>Cicha Noc (Metal Riff)</t>
-  </si>
-  <si>
     <t>RIFF</t>
   </si>
   <si>
+    <t>https://youtu.be/ZxoHOxQM_r8?si=QjNtVeNaQDZ09s6k</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1QI5mxWleqDsG0wNRaIdNIwffVb_JRe4o</t>
   </si>
   <si>
@@ -102,6 +105,9 @@
     <t>FINGERSTYLE</t>
   </si>
   <si>
+    <t>https://youtu.be/upT2NDOSrGI?si=rx0HOssBl1-TFxxp</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/0B-ZsE-2yneXrYmZKcVg2Z2tGM0E?resourcekey=0-5GyEuHBCKP1niL94OS8oxg</t>
   </si>
   <si>
@@ -114,6 +120,9 @@
     <t>Cicha Noc G dur</t>
   </si>
   <si>
+    <t>https://youtu.be/cS6I752ABKs?si=D3K570fFFHAFyFm3</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1Vk76zhGN7AwPFbfexHba2wrUsgVuPJzQ</t>
   </si>
   <si>
@@ -123,6 +132,9 @@
     <t>Deck the Halls</t>
   </si>
   <si>
+    <t>https://youtu.be/_Zws_4duo3I?si=lt4Zpna5Rvy-5Ca7</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/0B-ZsE-2yneXrdm8wRG5MaUpuT3M?resourcekey=0-R3OjDxpsbqtKhy7um-4Axg</t>
   </si>
   <si>
@@ -150,21 +162,21 @@
     <t>https://drive.google.com/drive/folders/0B-ZsE-2yneXrSjhBeFBsQ3ROWnc?resourcekey=0-Nbk10ztWR67kLJwXenFszw</t>
   </si>
   <si>
+    <t>https://youtu.be/T5eCKUw8dYE?si=KlTubtE0PzTxlY9N</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1GBwUaxrlZoH6GFgtWvY2r9wVjAwkFaLM</t>
   </si>
   <si>
-    <t>Dzisiaj W Betlejem (Gitara Elektryczna Solo)</t>
-  </si>
-  <si>
-    <t>SOLÓWKA</t>
-  </si>
-  <si>
     <t>https://drive.google.com/drive/folders/1dCrW9o0mDY6RwXtLK1PVtZZfBAkrBly_</t>
   </si>
   <si>
     <t>Dzisiaj W Betlejem G Dur</t>
   </si>
   <si>
+    <t>https://youtu.be/oWAq-0gXWjU?si=Rf3qGD3ACMb4ndws</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1ZIHq3uA4yYIjAadXXuYj4kgoRyIvuN7G</t>
   </si>
   <si>
@@ -183,18 +195,21 @@
     <t>Gdy Śliczna Panna</t>
   </si>
   <si>
+    <t>https://youtu.be/rzgk3j_DCjs?si=-mzNAuD5PRMaOF28</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1IXTRUMlLEMLOcJdNyT3cSBnMvayriWi4</t>
   </si>
   <si>
-    <t>Gdy Śliczna Panna (Gitara Elektryczna Solo)</t>
-  </si>
-  <si>
     <t>https://drive.google.com/drive/folders/1kaKhMQvFRMHA2Qdha4kpV3mwYj3dgZux</t>
   </si>
   <si>
     <t>Gdy Śliczna Panna G Dur</t>
   </si>
   <si>
+    <t>https://youtu.be/KDuyzulcci0?si=l3ftH3-6V-ZRr6YF</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1WNRmi39k3mUEkiDV9Gr6eWlVmpOY5nn8</t>
   </si>
   <si>
@@ -210,6 +225,9 @@
     <t>Jezus Malusieńki A Moll</t>
   </si>
   <si>
+    <t>https://youtu.be/8znwS6HvAEI?si=5Z6y95mRJRGLfyGg</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1kjoWdRJODsQ0xCubXPaNB6FMUmtnU_xw</t>
   </si>
   <si>
@@ -225,21 +243,33 @@
     <t>Jingle Bells</t>
   </si>
   <si>
+    <t>https://youtu.be/ASgM0aUBG38?si=SMHCF64_tXm-_P4a</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/0B-ZsE-2yneXrZ1dacmg5cXVOcms?resourcekey=0-XkwX97EDd5pMDwcSuDuVjQ</t>
   </si>
   <si>
+    <t>https://youtu.be/Zf9UqOuvG7A?si=UvXQ5U9YJYFaels5</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1oC4K3sWjSKe2ya0_efOI5tGLcxlNkpY3</t>
   </si>
   <si>
     <t>Jingle Bells G Dur</t>
   </si>
   <si>
+    <t>https://youtu.be/41GCnTQU7-g?si=0G6sTJXTLw_P211D</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1WgNezNv2ZScYIfTUHt0nEqEds-QA0_m7</t>
   </si>
   <si>
     <t>Last Christmas</t>
   </si>
   <si>
+    <t>https://youtu.be/1chaUEgzgR0?si=Ns33vOLtbbpEZMkG</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/0B-ZsE-2yneXrN3FJYTJldmVpelk?resourcekey=0-gbP_0zkPIb2GscepXmPbEw</t>
   </si>
   <si>
@@ -261,9 +291,15 @@
     <t>Lulajże Jezuniu D Dur</t>
   </si>
   <si>
+    <t>https://youtu.be/NzzE00CKN0o?si=j0Gbw5-76lRZTG5F</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1_F6a2ZhVfCe8YncYOgAMreOC4y3fR_ok</t>
   </si>
   <si>
+    <t>https://youtu.be/tMVIhU68AQU?si=yJp7JnAt3byvO-Sd</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1HsrRO41FJS8r0DIlB2wGVXDYKID9Zbve</t>
   </si>
   <si>
@@ -282,15 +318,18 @@
     <t>Pójdźmy Wszyscy Do Stajenki</t>
   </si>
   <si>
+    <t>https://youtu.be/LzgG-Jpeo0k?si=88du8w2fLUT-BU4Z</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1pF2XYa2xz6b8yGusD3S1XeatSV6HyZ_C</t>
   </si>
   <si>
+    <t>https://youtu.be/iAoMgqsoq3o?si=C7MjRAZAYFBi2uvx</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1DSQFzS1BvUyq7ric5WcqZSwhEhJ31mew</t>
   </si>
   <si>
-    <t>Pójdźmy Wszyscy Do Stajenki (Na jednej strunie)</t>
-  </si>
-  <si>
     <t>PROSTY</t>
   </si>
   <si>
@@ -306,27 +345,33 @@
     <t>https://drive.google.com/drive/folders/1X6Mws_fPx7Vb2SxV1Q0TlsY98qnCBMJz</t>
   </si>
   <si>
-    <t>Przybieżeli Do Betlejem (Na jednej strunie)</t>
-  </si>
-  <si>
     <t>https://drive.google.com/drive/folders/1eNyEOPqxYMJ5yd2KBWBaomPKiO3Ck9by</t>
   </si>
   <si>
     <t>Przybieżeli Do Betlejem C Dur</t>
   </si>
   <si>
+    <t>https://youtu.be/PfVSeNL8DBk?si=Bwu6oT6y1v6ckM8Z</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/0B-ZsE-2yneXrS2NRY1pIQ0g5UWc?resourcekey=0-OmQnBnwwHJHx4WmdiC4x9w</t>
   </si>
   <si>
     <t>Przybieżeli Do Betlejem G Dur</t>
   </si>
   <si>
+    <t>https://youtu.be/XZTnFhYnl08?si=wmMBrv7B74h732B0</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/1Xa4uWCRWqi_4PHT73jDs2UJtB_amoKhZ</t>
   </si>
   <si>
     <t>We Wish You a Merry Christmas C Dur</t>
   </si>
   <si>
+    <t>https://youtu.be/Dnd7oq9Fkmc?si=wLw86bhq9aJXVmjQ</t>
+  </si>
+  <si>
     <t>https://drive.google.com/drive/folders/0B-ZsE-2yneXrVUliTDBXRlMydWs?resourcekey=0-0S8bxoKqTFchrXXXeO7JBg</t>
   </si>
   <si>
@@ -348,70 +393,19 @@
     <t>https://drive.google.com/drive/folders/1ds3yHvAn526lOwvmVAbQeGguwhr_Ginr</t>
   </si>
   <si>
-    <t>https://youtu.be/XZTnFhYnl08?si=wmMBrv7B74h732B0</t>
-  </si>
-  <si>
-    <t>https://youtu.be/NzzE00CKN0o?si=j0Gbw5-76lRZTG5F</t>
-  </si>
-  <si>
-    <t>https://youtu.be/41GCnTQU7-g?si=0G6sTJXTLw_P211D</t>
-  </si>
-  <si>
-    <t>https://youtu.be/KDuyzulcci0?si=l3ftH3-6V-ZRr6YF</t>
-  </si>
-  <si>
-    <t>https://youtu.be/oWAq-0gXWjU?si=Rf3qGD3ACMb4ndws</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Zf9UqOuvG7A?si=UvXQ5U9YJYFaels5</t>
-  </si>
-  <si>
-    <t>https://youtu.be/ZxoHOxQM_r8?si=QjNtVeNaQDZ09s6k</t>
-  </si>
-  <si>
-    <t>https://youtu.be/cS6I752ABKs?si=D3K570fFFHAFyFm3</t>
-  </si>
-  <si>
-    <t>https://youtu.be/LzgG-Jpeo0k?si=88du8w2fLUT-BU4Z</t>
-  </si>
-  <si>
-    <t>https://youtu.be/iAoMgqsoq3o?si=C7MjRAZAYFBi2uvx</t>
-  </si>
-  <si>
-    <t>https://youtu.be/tMVIhU68AQU?si=yJp7JnAt3byvO-Sd</t>
-  </si>
-  <si>
-    <t>https://youtu.be/T5eCKUw8dYE?si=KlTubtE0PzTxlY9N</t>
-  </si>
-  <si>
-    <t>https://youtu.be/8znwS6HvAEI?si=5Z6y95mRJRGLfyGg</t>
-  </si>
-  <si>
-    <t>https://youtu.be/rzgk3j_DCjs?si=-mzNAuD5PRMaOF28</t>
-  </si>
-  <si>
-    <t>https://youtu.be/_Zws_4duo3I?si=lt4Zpna5Rvy-5Ca7</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Dnd7oq9Fkmc?si=wLw86bhq9aJXVmjQ</t>
-  </si>
-  <si>
-    <t>https://youtu.be/ASgM0aUBG38?si=SMHCF64_tXm-_P4a</t>
-  </si>
-  <si>
-    <t>https://youtu.be/PfVSeNL8DBk?si=Bwu6oT6y1v6ckM8Z</t>
-  </si>
-  <si>
-    <t>https://youtu.be/1chaUEgzgR0?si=Ns33vOLtbbpEZMkG</t>
-  </si>
-  <si>
-    <t>https://youtu.be/upT2NDOSrGI?si=rx0HOssBl1-TFxxp</t>
-  </si>
-  <si>
-    <t>BANALNY</t>
-  </si>
-  <si>
-    <t>ŚREDNI</t>
+    <t>TRUDNY</t>
+  </si>
+  <si>
+    <t>MELODIA</t>
+  </si>
+  <si>
+    <t>Przybieżeli Do Betlejem</t>
+  </si>
+  <si>
+    <t>Cicha Noc</t>
+  </si>
+  <si>
+    <t>SOLO</t>
   </si>
 </sst>
 </file>
@@ -431,7 +425,6 @@
       <name val="Carlito"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Carlito"/>
@@ -439,20 +432,16 @@
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
-      <charset val="238"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0563C1"/>
       <name val="Carlito"/>
-      <charset val="238"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Carlito"/>
-      <charset val="238"/>
     </font>
   </fonts>
   <fills count="2">
@@ -492,25 +481,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hiperłącze" xfId="2" builtinId="8"/>
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Hiperłącze" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
     <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="238"/>
-      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -530,21 +516,95 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="238"/>
-      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="238"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
         <left/>
         <right style="thin">
           <color indexed="64"/>
         </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left/>
+        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -555,10 +615,13 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <charset val="238"/>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF0563C1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -575,12 +638,20 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <charset val="238"/>
+        <u val="none"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -590,137 +661,7 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF0563C1"/>
-        <name val="Carlito"/>
-        <charset val="238"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="238"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="238"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Carlito"/>
-        <charset val="238"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="238"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <charset val="238"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -749,19 +690,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Baza__WI_TECZNE" displayName="Baza__WI_TECZNE" ref="A1:J50" totalsRowShown="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Baza__WI_TECZNE" displayName="Baza__WI_TECZNE" ref="A1:J50" totalsRowShown="0">
   <autoFilter ref="A1:J50" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="UTWÓR" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="POZIOM" dataDxfId="0" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="RODZAJ OPRACOWANIA" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="YOUTUBE" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="WYKONAWCA" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="KATEGORIE DODATKOWE" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="LINK DO DYSKU" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="OPIS" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="TAGI" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="DATA" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="UTWÓR" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="WYKONAWCA" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="POZIOM" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="RODZAJ OPRACOWANIA" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="KATEGORIE DODATKOWE" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="YOUTUBE" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="LINK DO DYSKU" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="OPIS" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="TAGI" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="DATA" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -962,22 +903,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="41.125" customWidth="1"/>
-    <col min="2" max="2" width="16.25" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="56.875" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="20.125" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="11" max="11" width="90" customWidth="1"/>
-    <col min="12" max="12" width="24.125" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="15" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="64" customWidth="1"/>
-    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="2" max="2" width="23.5" customWidth="1"/>
+    <col min="3" max="3" width="16.875" customWidth="1"/>
+    <col min="4" max="4" width="17.75" customWidth="1"/>
+    <col min="5" max="5" width="14.375" customWidth="1"/>
+    <col min="6" max="6" width="59.875" customWidth="1"/>
+    <col min="7" max="7" width="103.375" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="20.125" customWidth="1"/>
+    <col min="12" max="12" width="52" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="16" max="16" width="90" customWidth="1"/>
+    <col min="17" max="17" width="24.125" customWidth="1"/>
+    <col min="19" max="19" width="24" customWidth="1"/>
+    <col min="20" max="20" width="12" customWidth="1"/>
+    <col min="21" max="21" width="64" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -985,28 +930,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" t="s">
-        <v>4</v>
       </c>
       <c r="J1" t="s">
         <v>9</v>
@@ -1016,17 +961,17 @@
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>127</v>
-      </c>
+      <c r="B2" s="1"/>
       <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D2" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1"/>
       <c r="G2" s="3" t="s">
         <v>13</v>
       </c>
@@ -1038,19 +983,19 @@
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>128</v>
-      </c>
+      <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1"/>
       <c r="G3" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -1058,21 +1003,21 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>127</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="1"/>
       <c r="G4" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -1080,45 +1025,45 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>128</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="1"/>
       <c r="G5" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="4"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>128</v>
-      </c>
+      <c r="A6" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1" t="s">
-        <v>12</v>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -1126,23 +1071,23 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>128</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E7" s="1"/>
+        <v>25</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F7" s="1" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -1150,21 +1095,21 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>127</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="1"/>
       <c r="G8" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -1172,23 +1117,23 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>128</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="E9" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F9" s="1" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -1196,21 +1141,21 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>127</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="1"/>
       <c r="G10" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -1218,23 +1163,23 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>127</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E11" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F11" s="1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -1242,21 +1187,21 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>128</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B12" s="1"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="1"/>
       <c r="G12" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -1264,19 +1209,21 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="1"/>
       <c r="G13" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -1284,19 +1231,21 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="1"/>
       <c r="G14" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -1304,19 +1253,21 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="1"/>
       <c r="G15" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -1324,41 +1275,45 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="E16" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F16" s="1" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="4"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="2" t="s">
-        <v>42</v>
+      <c r="A17" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="1"/>
       <c r="G17" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -1366,21 +1321,23 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E18" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F18" s="1" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -1388,19 +1345,21 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D19" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="1"/>
       <c r="G19" s="3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -1408,19 +1367,21 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D20" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="1"/>
       <c r="G20" s="3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -1428,41 +1389,45 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E21" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F21" s="1" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="4"/>
     </row>
     <row r="22" spans="1:10">
-      <c r="A22" s="2" t="s">
-        <v>53</v>
+      <c r="A22" s="6" t="s">
+        <v>55</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="1"/>
       <c r="G22" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -1470,21 +1435,23 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E23" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F23" s="1" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
@@ -1492,19 +1459,21 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D24" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="1"/>
       <c r="G24" s="3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -1512,19 +1481,21 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="1"/>
       <c r="G25" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -1532,21 +1503,23 @@
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E26" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F26" s="1" t="s">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
@@ -1554,19 +1527,21 @@
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D27" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="1"/>
       <c r="G27" s="3" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -1574,19 +1549,21 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="1"/>
       <c r="G28" s="3" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
@@ -1594,7 +1571,7 @@
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B29" s="1"/>
       <c r="C29" s="1" t="s">
@@ -1603,12 +1580,14 @@
       <c r="D29" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E29" s="1"/>
+      <c r="E29" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F29" s="1" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -1616,21 +1595,23 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B30" s="1"/>
       <c r="C30" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E30" s="1"/>
+        <v>25</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
@@ -1638,21 +1619,23 @@
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="2" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B31" s="1"/>
       <c r="C31" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E31" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F31" s="1" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
@@ -1660,21 +1643,23 @@
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="2" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="B32" s="1"/>
       <c r="C32" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="E32" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F32" s="1" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
@@ -1682,19 +1667,21 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="2" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="B33" s="1"/>
       <c r="C33" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" s="1"/>
       <c r="G33" s="3" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
@@ -1702,19 +1689,21 @@
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="2" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B34" s="1"/>
       <c r="C34" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" s="1"/>
       <c r="G34" s="3" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
@@ -1722,19 +1711,21 @@
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="2" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B35" s="1"/>
       <c r="C35" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D35" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" s="1"/>
       <c r="G35" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
@@ -1742,21 +1733,23 @@
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B36" s="1"/>
       <c r="C36" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="E36" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F36" s="1" t="s">
-        <v>12</v>
+        <v>88</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
@@ -1764,21 +1757,23 @@
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B37" s="1"/>
       <c r="C37" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E37" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F37" s="1" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
@@ -1786,19 +1781,21 @@
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="2" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="B38" s="1"/>
       <c r="C38" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D38" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" s="1"/>
       <c r="G38" s="3" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
@@ -1806,19 +1803,21 @@
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="2" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="B39" s="1"/>
       <c r="C39" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D39" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" s="1"/>
       <c r="G39" s="3" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
@@ -1826,21 +1825,23 @@
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="2" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="B40" s="1"/>
       <c r="C40" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="E40" s="1"/>
+        <v>25</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F40" s="1" t="s">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
@@ -1848,43 +1849,45 @@
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="2" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="B41" s="1"/>
       <c r="C41" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E41" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F41" s="1" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
       <c r="J41" s="4"/>
     </row>
     <row r="42" spans="1:10">
-      <c r="A42" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>88</v>
-      </c>
+      <c r="A42" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B42" s="1"/>
       <c r="C42" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42" s="1"/>
       <c r="G42" s="3" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
@@ -1892,41 +1895,43 @@
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="2" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="B43" s="1"/>
       <c r="C43" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D43" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F43" s="1"/>
       <c r="G43" s="3" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
       <c r="J43" s="4"/>
     </row>
     <row r="44" spans="1:10">
-      <c r="A44" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>88</v>
-      </c>
+      <c r="A44" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B44" s="1"/>
       <c r="C44" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F44" s="1"/>
       <c r="G44" s="3" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
@@ -1934,21 +1939,23 @@
     </row>
     <row r="45" spans="1:10">
       <c r="A45" s="2" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B45" s="1"/>
       <c r="C45" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="E45" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F45" s="1" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
@@ -1956,21 +1963,23 @@
     </row>
     <row r="46" spans="1:10">
       <c r="A46" s="2" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B46" s="1"/>
       <c r="C46" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E46" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F46" s="1" t="s">
-        <v>12</v>
+        <v>111</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
@@ -1978,21 +1987,23 @@
     </row>
     <row r="47" spans="1:10">
       <c r="A47" s="2" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="B47" s="1"/>
       <c r="C47" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E47" s="1"/>
+        <v>123</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>12</v>
+      </c>
       <c r="F47" s="1" t="s">
-        <v>12</v>
+        <v>114</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
@@ -2000,19 +2011,21 @@
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="2" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="B48" s="1"/>
       <c r="C48" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D48" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F48" s="1"/>
       <c r="G48" s="3" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
@@ -2020,19 +2033,21 @@
     </row>
     <row r="49" spans="1:10">
       <c r="A49" s="2" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="B49" s="1"/>
       <c r="C49" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D49" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F49" s="1"/>
       <c r="G49" s="3" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
@@ -2040,19 +2055,21 @@
     </row>
     <row r="50" spans="1:10">
       <c r="A50" s="2" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="B50" s="1"/>
       <c r="C50" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
-      <c r="F50" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D50" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F50" s="1"/>
       <c r="G50" s="3" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
@@ -2060,12 +2077,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D6" r:id="rId1" xr:uid="{C43855BC-8253-4BA7-8C6D-C57C089E7402}"/>
+    <hyperlink ref="F6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>